<commit_message>
feat: replace template Excel file with updated version from Downloads
</commit_message>
<xml_diff>
--- a/public/templates/NNP_QL_HO_SO_PHUONG_TIEN_CANG.xlsx
+++ b/public/templates/NNP_QL_HO_SO_PHUONG_TIEN_CANG.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVPL-NgocAnh\Desktop\Tools\BAOCAOCANHANG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVPL-NgocAnh\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE318482-F1EE-4FB9-AC06-CB305EA572B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F72D3F7A-3C59-4BBA-8DD7-E69F703075DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hồ sơ phương tiện" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="85">
   <si>
     <t>STT</t>
   </si>
@@ -157,6 +157,9 @@
     <t>Nguyễn Quốc Dũng</t>
   </si>
   <si>
+    <t>Viên Nén Gỗ</t>
+  </si>
+  <si>
     <t>Trạng Thái Thuyền Viên</t>
   </si>
   <si>
@@ -193,12 +196,18 @@
     <t>14473/ĐK</t>
   </si>
   <si>
+    <t>VR-SII</t>
+  </si>
+  <si>
     <t>Nguyễn Quốc Toàn</t>
   </si>
   <si>
     <t>Lữ Thị Kiều Trang</t>
   </si>
   <si>
+    <t>Nguyễn Trường Thoại</t>
+  </si>
+  <si>
     <t>Không</t>
   </si>
   <si>
@@ -281,24 +290,17 @@
   </si>
   <si>
     <t>Lê Vinh</t>
-  </si>
-  <si>
-    <t>V63-12714</t>
-  </si>
-  <si>
-    <t>Nguyễn Hoài Hận</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,19 +338,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="163"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,30 +359,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -418,10 +390,10 @@
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -443,55 +415,16 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -849,15 +782,15 @@
     <col min="2" max="2" width="23.77734375" style="1" customWidth="1"/>
     <col min="3" max="3" width="15.44140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" style="16" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" style="16" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" style="16" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" style="20" customWidth="1"/>
-    <col min="9" max="9" width="13.21875" style="20" customWidth="1"/>
-    <col min="10" max="10" width="17.21875" style="20" customWidth="1"/>
-    <col min="11" max="11" width="14.77734375" style="25" customWidth="1"/>
-    <col min="12" max="12" width="13.21875" style="25" customWidth="1"/>
-    <col min="13" max="13" width="13.77734375" style="25" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="13.21875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="17.21875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.77734375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" style="5" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" style="5" customWidth="1"/>
     <col min="14" max="14" width="9.44140625" style="5" customWidth="1"/>
     <col min="15" max="15" width="16.88671875" style="5" customWidth="1"/>
     <col min="16" max="16" width="15.44140625" style="5" customWidth="1"/>
@@ -887,31 +820,31 @@
       <c r="D1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="L1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="N1" s="3" t="s">
@@ -945,10 +878,10 @@
         <v>19</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Z1" s="3" t="s">
         <v>4</v>
@@ -968,31 +901,31 @@
       <c r="D2" s="4">
         <v>400</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="8">
         <v>42893</v>
       </c>
-      <c r="G2" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H2" s="19" t="s">
+      <c r="G2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="19">
+      <c r="I2" s="8">
         <v>46174</v>
       </c>
-      <c r="J2" s="19">
+      <c r="J2" s="8">
         <v>46532</v>
       </c>
-      <c r="K2" s="23">
+      <c r="K2" s="9">
         <v>8154841</v>
       </c>
-      <c r="L2" s="24">
+      <c r="L2" s="8">
         <v>46168</v>
       </c>
-      <c r="M2" s="24">
+      <c r="M2" s="8">
         <v>46538</v>
       </c>
       <c r="N2" s="4" t="str">
@@ -1046,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" s="7">
         <v>1290</v>
@@ -1054,31 +987,31 @@
       <c r="D3" s="4">
         <v>380</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="15">
+      <c r="E3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="8">
         <v>42433</v>
       </c>
-      <c r="G3" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="19">
+      <c r="G3" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="8">
         <v>46108</v>
       </c>
-      <c r="J3" s="19">
+      <c r="J3" s="8">
         <v>46473</v>
       </c>
-      <c r="K3" s="22">
+      <c r="K3" s="4">
         <v>7342177</v>
       </c>
-      <c r="L3" s="24">
+      <c r="L3" s="8">
         <v>46210</v>
       </c>
-      <c r="M3" s="24">
+      <c r="M3" s="8">
         <v>46575</v>
       </c>
       <c r="N3" s="4" t="str">
@@ -1098,21 +1031,21 @@
         <v>CÒN HẠN</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S3" s="4" t="str">
         <f t="shared" ref="S3:S8" si="5">IF(C3&gt;1000,"T1",IF(C3&gt;=500,"T2","T3"))</f>
         <v>T1</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="U3" s="4" t="str">
         <f t="shared" ref="U3:U8" si="6">IF(D3&lt;=250,"M3",IF(D3&lt;=1000,"M2","M1"))</f>
         <v>M2</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W3" s="4" t="s">
         <v>38</v>
@@ -1132,7 +1065,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="7">
         <v>1618</v>
@@ -1140,36 +1073,28 @@
       <c r="D4" s="4">
         <v>385</v>
       </c>
-      <c r="E4" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="15">
+      <c r="E4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="8">
         <v>43131</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" s="19">
-        <v>46048</v>
-      </c>
-      <c r="J4" s="19">
-        <v>46413</v>
-      </c>
-      <c r="K4" s="22">
-        <v>6437238</v>
-      </c>
-      <c r="L4" s="24">
-        <v>46200</v>
-      </c>
-      <c r="M4" s="24">
-        <v>46382</v>
-      </c>
+      <c r="G4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="8">
+        <v>46768</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
       <c r="N4" s="4" t="str">
-        <f>IF(AND(E4&lt;&gt;"",H4&lt;&gt;"",K4&lt;&gt;""),"ĐỦ","THIẾU")</f>
-        <v>ĐỦ</v>
+        <f t="shared" si="1"/>
+        <v>THIẾU</v>
       </c>
       <c r="O4" s="4" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1181,31 +1106,31 @@
       </c>
       <c r="Q4" s="4" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>CÒN HẠN</v>
+        <v/>
       </c>
       <c r="R4" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="S4" s="4" t="str">
         <f t="shared" si="5"/>
         <v>T1</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="U4" s="4" t="str">
         <f t="shared" si="6"/>
         <v>M2</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="X4" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>PHÙ HỢP</v>
+        <v>KHÔNG PHÙ HỢP</v>
       </c>
       <c r="Y4" s="4" t="s">
         <v>38</v>
@@ -1218,7 +1143,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C5" s="7">
         <v>1600</v>
@@ -1226,31 +1151,31 @@
       <c r="D5" s="4">
         <v>380</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" s="15">
+      <c r="E5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="8">
         <v>42503</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="I5" s="19">
+      <c r="G5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="8">
         <v>45937</v>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="8">
         <v>46277</v>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="4">
         <v>7731971</v>
       </c>
-      <c r="L5" s="24">
+      <c r="L5" s="8">
         <v>46292</v>
       </c>
-      <c r="M5" s="24">
+      <c r="M5" s="8">
         <v>46292</v>
       </c>
       <c r="N5" s="4" t="str">
@@ -1270,21 +1195,21 @@
         <v>CÒN HẠN</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="S5" s="4" t="str">
         <f t="shared" si="5"/>
         <v>T1</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="U5" s="4" t="str">
         <f t="shared" si="6"/>
         <v>M2</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="W5" s="4" t="s">
         <v>38</v>
@@ -1294,7 +1219,7 @@
         <v>PHÙ HỢP</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Z5" s="4"/>
     </row>
@@ -1304,7 +1229,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C6" s="7">
         <v>1600</v>
@@ -1312,31 +1237,31 @@
       <c r="D6" s="4">
         <v>400</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F6" s="15">
+      <c r="E6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="8">
         <v>42887</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="I6" s="19">
+      <c r="G6" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I6" s="8">
         <v>46178</v>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="8">
         <v>46533</v>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="4">
         <v>8154768</v>
       </c>
-      <c r="L6" s="24">
+      <c r="L6" s="8">
         <v>46173</v>
       </c>
-      <c r="M6" s="24">
+      <c r="M6" s="8">
         <v>46537</v>
       </c>
       <c r="N6" s="4" t="str">
@@ -1356,21 +1281,21 @@
         <v>CÒN HẠN</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="S6" s="4" t="str">
         <f t="shared" si="5"/>
         <v>T1</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="U6" s="4" t="str">
         <f t="shared" si="6"/>
         <v>M2</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="W6" s="4" t="s">
         <v>38</v>
@@ -1380,7 +1305,7 @@
         <v>PHÙ HỢP</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Z6" s="4"/>
     </row>
@@ -1390,7 +1315,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C7" s="7">
         <v>1995</v>
@@ -1398,31 +1323,31 @@
       <c r="D7" s="4">
         <v>385</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" s="15">
+      <c r="E7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="8">
         <v>43139</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="I7" s="19">
+      <c r="G7" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" s="8">
         <v>46066</v>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="8">
         <v>46430</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="4">
         <v>7977931</v>
       </c>
-      <c r="L7" s="24">
+      <c r="L7" s="8">
         <v>46059</v>
       </c>
-      <c r="M7" s="24">
+      <c r="M7" s="8">
         <v>46438</v>
       </c>
       <c r="N7" s="4" t="str">
@@ -1442,21 +1367,21 @@
         <v>CÒN HẠN</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="S7" s="4" t="str">
         <f t="shared" si="5"/>
         <v>T1</v>
       </c>
       <c r="T7" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="U7" s="4" t="str">
         <f t="shared" si="6"/>
         <v>M2</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="W7" s="4" t="s">
         <v>38</v>
@@ -1466,7 +1391,7 @@
         <v>PHÙ HỢP</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Z7" s="4"/>
     </row>
@@ -1476,7 +1401,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C8" s="7">
         <v>1200</v>
@@ -1484,31 +1409,31 @@
       <c r="D8" s="4">
         <v>355</v>
       </c>
-      <c r="E8" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="15">
+      <c r="E8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="8">
         <v>43732</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="I8" s="19">
+      <c r="G8" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I8" s="8">
         <v>45967</v>
       </c>
-      <c r="J8" s="19">
+      <c r="J8" s="8">
         <v>46331</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="4">
         <v>7975404</v>
       </c>
-      <c r="L8" s="24">
+      <c r="L8" s="8">
         <v>46058</v>
       </c>
-      <c r="M8" s="24">
+      <c r="M8" s="8">
         <v>46438</v>
       </c>
       <c r="N8" s="4" t="str">
@@ -1528,21 +1453,21 @@
         <v>CÒN HẠN</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="S8" s="4" t="str">
         <f t="shared" si="5"/>
         <v>T1</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="U8" s="4" t="str">
         <f t="shared" si="6"/>
         <v>M2</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="W8" s="4" t="s">
         <v>38</v>
@@ -1586,18 +1511,18 @@
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="20" style="4" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="17.77734375" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="19.5546875" style="4" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.5546875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="8.77734375" style="2"/>
   </cols>
   <sheetData>
@@ -1606,13 +1531,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>21</v>
@@ -1647,13 +1572,13 @@
       <c r="B2" s="8">
         <v>46212</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="10">
         <v>0.9604166666666667</v>
       </c>
       <c r="D2" s="8">
         <v>46213</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="10">
         <v>0.86805555555555558</v>
       </c>
       <c r="F2" s="4" t="s">
@@ -1663,9 +1588,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(F2,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>5785/ĐK</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>62</v>
-      </c>
+      <c r="H2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="4"/>
       <c r="J2" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F2,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1687,25 +1613,26 @@
       <c r="B3" s="8">
         <v>46213</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>0.68055555555555558</v>
       </c>
       <c r="D3" s="8">
         <v>46214</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="10">
         <v>0.57638888888888884</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G3" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F3,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>14008/ĐK</v>
       </c>
-      <c r="H3" s="10" t="s">
-        <v>62</v>
-      </c>
+      <c r="H3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="4"/>
       <c r="J3" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F3,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1727,36 +1654,37 @@
       <c r="B4" s="8">
         <v>46214</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>0.11597222222222223</v>
       </c>
       <c r="D4" s="8">
-        <v>46217</v>
-      </c>
-      <c r="E4" s="9">
-        <v>0.58273148148148146</v>
+        <v>46216</v>
+      </c>
+      <c r="E4" s="10">
+        <v>0.6386574074074074</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G4" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>14473/ĐK</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>49</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="I4" s="4"/>
       <c r="J4" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
-        <v>ĐỦ</v>
+        <v>THIẾU</v>
       </c>
       <c r="K4" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$X:$X),"")</f>
-        <v>PHÙ HỢP</v>
+        <v>KHÔNG PHÙ HỢP</v>
       </c>
       <c r="L4" s="4" t="str">
         <f>IF(AND(J4="Đủ",K4="PHÙ HỢP"),"CHO PHÉP","KHÔNG CHO PHÉP")</f>
-        <v>CHO PHÉP</v>
+        <v>KHÔNG CHO PHÉP</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1767,25 +1695,26 @@
       <c r="B5" s="8">
         <v>46214</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>0.4826388888888889</v>
       </c>
       <c r="D5" s="8">
         <v>46215</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="10">
         <v>0.35606481481481483</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G5" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F5,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>1803/ĐK</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I5" s="4"/>
       <c r="J5" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F5,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1807,25 +1736,26 @@
       <c r="B6" s="8">
         <v>46215</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>0.32847222222222222</v>
       </c>
       <c r="D6" s="8">
         <v>46216</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="10">
         <v>0.36038194444444444</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G6" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F6,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>6537/ĐK</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I6" s="4"/>
       <c r="J6" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F6,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1847,25 +1777,26 @@
       <c r="B7" s="8">
         <v>46216</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>0.39583333333333331</v>
       </c>
       <c r="D7" s="8">
         <v>46217</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="10">
         <v>0.68472222222222223</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G7" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F7,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>1554/ĐK</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I7" s="4"/>
       <c r="J7" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F7,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1887,25 +1818,22 @@
       <c r="B8" s="8">
         <v>46216</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="10">
         <v>0.90277777777777779</v>
       </c>
-      <c r="D8" s="8">
-        <v>46217</v>
-      </c>
-      <c r="E8" s="9">
-        <v>0.6875</v>
-      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G8" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F8,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$E:$E),"")</f>
         <v>8604/ĐK</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I8" s="4"/>
       <c r="J8" s="4" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F8,'Hồ sơ phương tiện'!$B:$B,'Hồ sơ phương tiện'!$N:$N),"")</f>
         <v>ĐỦ</v>
@@ -1952,26 +1880,26 @@
       </c>
       <c r="B1" s="12"/>
     </row>
-    <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B2" s="6">
         <f>COUNTIF('Hồ sơ phương tiện'!N:N,"ĐỦ")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B3" s="6">
         <f>COUNTIF('Hồ sơ phương tiện'!N:N,"THIẾU")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B4" s="6">

</xml_diff>

<commit_message>
feat: strip Excel conditional formatting from template and apply static yellow styling for Sheet 1 (N, X) and Sheet 2 (J, L) when values are incomplete/incorrect
</commit_message>
<xml_diff>
--- a/public/templates/NNP_QL_HO_SO_PHUONG_TIEN_CANG.xlsx
+++ b/public/templates/NNP_QL_HO_SO_PHUONG_TIEN_CANG.xlsx
@@ -1482,21 +1482,6 @@
       <c r="Z8" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="N1:N1048576">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
-      <formula>"THIẾU"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X1:X1048576">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
-      <formula>"KHÔNG PHÙ HỢP"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y1:Y1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
-      <formula>"Không"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="Y2:Y8 W2:W8" xr:uid="{584CE58A-6625-4A71-80DC-3BB9FBC87D42}">
       <formula1>"Có,Không"</formula1>
@@ -1848,19 +1833,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"KHÔNG PHÙ HỢP"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L1:L1048576">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"KHÔNG CHO PHÉP"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>"KHÔNG ĐỦ HỒ SƠ"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>